<commit_message>
P-2026-0046 REV. 3: Quitar partida 02 zapatas/anclajes (a cargo constructor) y partida 05 cables
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0046-estructura-cubo-inox-lacado-blanco-binibeca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0046-estructura-cubo-inox-lacado-blanco-binibeca/presupuesto.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y VALORACIÓN ECONÓMICA: P-2026-0046 (REV. 2)</t>
+          <t>PRESUPUESTO TÉCNICO Y VALORACIÓN ECONÓMICA: P-2026-0046 (REV. 3)</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026 · Validez 30 días</t>
+          <t>30/10/2026 · Validez 30 días</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Estructura cúbica minimalista en tubo de Acero Inoxidable 40x40x2 mm lacado blanco, amurada al piso sin pernos vistos</t>
+          <t>Estructura cúbica minimalista en tubo de Acero Inoxidable 40x40x2 mm lacado blanco, fijada sobre zapatas ejecutadas por constructor</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Medidas: 4,00 x 3,00 x 2,50 m (12 m²) | Geometría cúbica ortoédrica | Tubo cuadrado de Acero Inoxidable 40x40x2 mm | Soldadura TIG pulida | Termolacado al horno en Blanco exterior (RAL 9010/9016) | Fijación amurada al piso mediante espigas macizas inox y anclaje químico (cero pernos salientes para caminar descalzo) | Costillas superiores y red tensada Inox AISI 316 para trepadoras</t>
+          <t>Medidas: 4,00 x 3,00 x 2,50 m (12 m²) | Geometría cúbica ortoédrica | Tubo cuadrado de Acero Inoxidable 40x40x2 mm | Soldadura TIG pulida | Termolacado al horno en Blanco exterior (RAL 9010/9016) | Obra civil y zapatas a cargo del constructor | Transporte y montaje de estructura fijada sobre puntos de obra</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Replanteo técnico in situ, nivelación y desarrollo de planos de taller: visita a Binibeca Vell para replanteo con D.F. y albañilería; cotas de solera e=10cm y cota cero porcelánico C3</t>
+          <t>Replanteo técnico in situ, nivelación y desarrollo de planos de taller: visita a la obra en Binibeca Vell para comprobación de cotas y coordinación de apoyos con el constructor previa ejecución de zapatas/solera, y elaboración de planos de taller</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Sistema de fijación oculta amurada al piso 'Pies Descalzos' (Fase 1 previa a solado): 4 espigas macizas inox Ø25 mm, vainas cilíndricas empotrables e inyección química de resina epoxi Fischer (superficie 100% enrasada bajo porcelánico C3, cero pernos salientes)</t>
+          <t>Fabricación en taller de estructura cúbica en tubo de Acero Inoxidable 40x40x2 mm: 4 pilares verticales de 2,50 m, marco perimetral superior (2 vigas de 4 m + 2 vigas de 3 m) y costillas intermedias superiores transversales de rigidización. Cortes ingleteados a 45º, soldadura continua TIG en atmósfera inerte de argón y aristas esmeriladas para acabado monolítico</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -671,7 +671,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>420</v>
+        <v>2150</v>
       </c>
       <c r="F14" s="12">
         <f>D14*E14</f>
@@ -686,7 +686,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Fabricación en taller de estructura cúbica en tubo de Acero Inoxidable 40x40x2 mm: 4 pilares h=2,50 m, marco perimetral superior (2 vigas 4m + 2 vigas 3m) y 4 costillas intermedias superiores transversales cada 80 cm. Cortes ingleteados 45º, soldadura continua TIG en argón y aristas esmeriladas</t>
+          <t>Tratamiento superficial de termolacado al horno en Blanco Exterior: desengrasado, acondicionamiento superficial para acero inoxidable, imprimación de adherencia técnica y termolacado al horno con pintura en polvo de resinas de poliéster arquitectónico (Blanco RAL 9010/9016) resistente a radiación UV y salinidad marina</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -698,7 +698,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>2150</v>
+        <v>680</v>
       </c>
       <c r="F15" s="12">
         <f>D15*E15</f>
@@ -713,7 +713,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Tratamiento superficial de termolacado al horno en Blanco Exterior: desengrasado, acondicionamiento superficial para inox, imprimación de adherencia y aplicación termolacada al horno con polvo poliéster arquitectónico (Blanco RAL 9010/9016) resistente a intemperie marina y UV</t>
+          <t>Transporte a Binibeca Vell y montaje de estructura sobre puntos preparados: transporte especializado a obra, descarga, elevación de módulos, aplomado y fijación estructural sobre los puntos/zapatas ejecutados por el constructor, verificación de niveles, repaso de lacado y retirada de embalajes</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -725,123 +725,69 @@
         <v>1</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>680</v>
+        <v>980</v>
       </c>
       <c r="F16" s="12">
         <f>D16*E16</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Entramado tensor de cables de acero inoxidable AISI 316 para trepadoras: retícula de cables 1x19 Ø3-4mm tensados entre las costillas de tubo 40x40 con tensores de botella náuticos A4 para soporte vegetal y resistencia al viento</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>lote</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>390</v>
-      </c>
-      <c r="F17" s="12">
-        <f>D17*E17</f>
+    <row r="18">
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Base Imponible:</t>
+        </is>
+      </c>
+      <c r="F18" s="13">
+        <f>SUM(F13:F16)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Transporte especializado a Binibeca Vell y montaje integral: entrega de vainas/esperas en Fase 1 y montaje completo de estructura modular en Fase 2, aplomado, inyección química al piso y limpieza final</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>lote</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>980</v>
-      </c>
-      <c r="F18" s="12">
-        <f>D18*E18</f>
+    <row r="19">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>IVA (21%):</t>
+        </is>
+      </c>
+      <c r="F19" s="14">
+        <f>F18*0.21</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL PRESUPUESTO:</t>
+        </is>
+      </c>
+      <c r="F20" s="15">
+        <f>F18+F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>VARIANTE ALTERNATIVA: Estructura Cúbica 4,00 x 2,00 m (8,00 m²)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Base Imponible:</t>
         </is>
       </c>
-      <c r="F20" s="13">
-        <f>SUM(F13:F18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>IVA (21%):</t>
-        </is>
-      </c>
-      <c r="F21" s="14">
-        <f>F20*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL PRESUPUESTO:</t>
-        </is>
-      </c>
-      <c r="F22" s="15">
-        <f>F20+F21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>VARIANTE ALTERNATIVA: Estructura Cúbica 4,00 x 2,00 m (8,00 m²)</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Base Imponible:</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>4180</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F22" s="13" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Total con IVA (21%):</t>
         </is>
       </c>
-      <c r="F25" s="13" t="n">
-        <v>5057.8</v>
+      <c r="F23" s="13" t="n">
+        <v>4235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>